<commit_message>
Prompt engineering almost complete. First draft batch API code created.
</commit_message>
<xml_diff>
--- a/Publications/GenAI/1_prompt_debugging/Specific_Boundary_Cases.xlsx
+++ b/Publications/GenAI/1_prompt_debugging/Specific_Boundary_Cases.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Edge Cases for Few-Shot" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="94">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -275,6 +276,12 @@
     <t xml:space="preserve">Agree with LLM, not in scope. Specifically focussed on animal feed, not human food.</t>
   </si>
   <si>
+    <t xml:space="preserve">This is a general consumer attitudes and food safety tracking survey with only incidental mention of cultivated meat as one awareness metric among many unrelated food concerns; it does not substantively research alternative proteins, their development, characterisation, or acceptance in ways that advance the field.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In scope. I can see the issue but not sure I can fix it… More edge case.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Important notes:</t>
   </si>
   <si>
@@ -288,6 +295,21 @@
   </si>
   <si>
     <t xml:space="preserve">I am similarly concerned about the exclusion for foods that do not substitute animal proteins (e.g. bread, pasta, snacks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pub.1186250605</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changing Food in a Changing World: Assessing Compliance to Insects, Cultivated Meat, and Soil-Less Products Among Italian Undergraduates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Background/Objectives: In recent decades, the need for sustainable alternatives to traditional foods for the global population has become urgent. To this aim, edible insects, cultivated meat, and vegetables produced through soil-less farming have been proposed. This cross-sectional study was aimed at exploring willingness to eat these novel foods and its possible correlates in young Italian adults. Methods: An electronic questionnaire was administered to the student populations of 13 universities throughout the Italian territory. Results: The results show that insects and cultivated meat were widely acknowledged as possible food, while soil-free cultivation seems to be less known. Indeed, the percentage of participants who have heard of insects, cultivated meat, and soil-free cultivation was respectively equal to 91.5%, 84.7%, and 32.9%. However, the majority of respondents were uncertain about the sustainability of all the proposed products (52.6% for insects, 39.5% for cultivated meat, and 58.0% for soil-free cultivation, respectively), and the propensity to try and eat insects (9.5%) was lower than that declared for synthetic meat (22.8%) and products from soil-free cultivation (19.2%). However, the regression analysis showed that the propensity to eat these foods regularly is positively related to the confidence in their sustainability (p &lt; 0.001). Willingness to try each of the proposed foods positively correlated with that declared for the others (p &lt; 0.001). Conclusions: These findings highlight the need to implement interventions aimed at increasing awareness about the use of these products as alternatives to less sustainable foods and the importance of identifying consumer groups to which these interventions should be addressed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">While cultivated meat is mentioned, the publication's primary focus is consumer acceptance and willingness to eat novel foods including insects (explicitly excluded), soil-less vegetables (not alternative proteins), and cultivated meat; the substantive content concerns broad dietary acceptance rather than advancing alternative protein development, characterisation, or understanding, making it primarily a general food acceptance study rather than alternative protein research.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concerning that it thinks I excluded consumer acceptance?</t>
   </si>
 </sst>
 </file>
@@ -329,7 +351,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -340,6 +362,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF81D41A"/>
+        <bgColor rgb="FF969696"/>
       </patternFill>
     </fill>
   </fills>
@@ -377,7 +405,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -422,6 +450,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -431,6 +463,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF81D41A"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1259,6 +1351,58 @@
       <c r="P12" s="9"/>
       <c r="Q12" s="9"/>
     </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="H17" s="3" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="J17" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="K17" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="N17" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="O17" s="0" t="s">
+        <v>83</v>
+      </c>
+    </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -1282,27 +1426,98 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A2:O2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="H2" s="3" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="M2" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="N2" s="4" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>